<commit_message>
Laminas comunales regeneradas: Educacion, Ocupacion, Pensiones y Salud desde la capa
Incluye las dos comunas que salian en blanco en todos los mapas comunales de
esas cuatro dimensiones: Paihuano y Marchigue ahora traen su valor.
</commit_message>
<xml_diff>
--- a/output/graficos_dimensiones/comunal_e_basbrut_a_2018_coquimbo.xlsx
+++ b/output/graficos_dimensiones/comunal_e_basbrut_a_2018_coquimbo.xlsx
@@ -87,7 +87,7 @@
     <t xml:space="preserve">Fecha de creación</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-09-10 00:23</t>
+    <t xml:space="preserve">2026-09-18 10:35</t>
   </si>
   <si>
     <t xml:space="preserve">Fuente</t>
@@ -757,8 +757,12 @@
       <c r="C16" s="2" t="n">
         <v>4105</v>
       </c>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
+      <c r="D16" s="2" t="n">
+        <v>2018</v>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>97.82</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:E16"/>

</xml_diff>